<commit_message>
trabajo de hoy 13 de abril de 2026
</commit_message>
<xml_diff>
--- a/2_ejecucion_plan_trabajo/2_consolidacion_datos_meteoro_epidemiologicos_reales/03_fusionados_y_limpieza_datos/df_final_fusionado.xlsx
+++ b/2_ejecucion_plan_trabajo/2_consolidacion_datos_meteoro_epidemiologicos_reales/03_fusionados_y_limpieza_datos/df_final_fusionado.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,94 +421,94 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>año</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>semana_epi</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>casos_dengue</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>temp</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>temp_max</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>temp_min</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>hum_esp</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>hum_rel</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>prec</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>dias_lluvia</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>vel_vi</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>vel_vi_max</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>vel_vi_min</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>uv</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>soi</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>sst</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>44199</v>
       </c>
       <c r="B2" t="n">
@@ -573,7 +561,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>44206</v>
       </c>
       <c r="B3" t="n">
@@ -626,7 +614,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>44213</v>
       </c>
       <c r="B4" t="n">
@@ -679,7 +667,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>44220</v>
       </c>
       <c r="B5" t="n">
@@ -732,7 +720,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>44227</v>
       </c>
       <c r="B6" t="n">
@@ -785,7 +773,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>44234</v>
       </c>
       <c r="B7" t="n">
@@ -838,7 +826,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>44241</v>
       </c>
       <c r="B8" t="n">
@@ -891,7 +879,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>44248</v>
       </c>
       <c r="B9" t="n">
@@ -944,7 +932,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>44255</v>
       </c>
       <c r="B10" t="n">
@@ -997,7 +985,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>44262</v>
       </c>
       <c r="B11" t="n">
@@ -1050,7 +1038,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>44269</v>
       </c>
       <c r="B12" t="n">
@@ -1103,7 +1091,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>44276</v>
       </c>
       <c r="B13" t="n">
@@ -1156,7 +1144,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>44283</v>
       </c>
       <c r="B14" t="n">
@@ -1209,7 +1197,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>44290</v>
       </c>
       <c r="B15" t="n">
@@ -1262,7 +1250,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>44297</v>
       </c>
       <c r="B16" t="n">
@@ -1315,7 +1303,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>44304</v>
       </c>
       <c r="B17" t="n">
@@ -1368,7 +1356,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>44311</v>
       </c>
       <c r="B18" t="n">
@@ -1421,7 +1409,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>44318</v>
       </c>
       <c r="B19" t="n">
@@ -1474,7 +1462,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>44325</v>
       </c>
       <c r="B20" t="n">
@@ -1527,7 +1515,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>44332</v>
       </c>
       <c r="B21" t="n">
@@ -1580,7 +1568,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>44339</v>
       </c>
       <c r="B22" t="n">
@@ -1633,7 +1621,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>44346</v>
       </c>
       <c r="B23" t="n">
@@ -1686,7 +1674,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>44353</v>
       </c>
       <c r="B24" t="n">
@@ -1739,7 +1727,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>44360</v>
       </c>
       <c r="B25" t="n">
@@ -1792,7 +1780,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>44367</v>
       </c>
       <c r="B26" t="n">
@@ -1845,7 +1833,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>44374</v>
       </c>
       <c r="B27" t="n">
@@ -1898,7 +1886,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>44381</v>
       </c>
       <c r="B28" t="n">
@@ -1951,7 +1939,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>44388</v>
       </c>
       <c r="B29" t="n">
@@ -2004,7 +1992,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>44395</v>
       </c>
       <c r="B30" t="n">
@@ -2057,7 +2045,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>44402</v>
       </c>
       <c r="B31" t="n">
@@ -2110,7 +2098,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>44409</v>
       </c>
       <c r="B32" t="n">
@@ -2163,7 +2151,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>44416</v>
       </c>
       <c r="B33" t="n">
@@ -2216,7 +2204,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>44423</v>
       </c>
       <c r="B34" t="n">
@@ -2269,7 +2257,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>44430</v>
       </c>
       <c r="B35" t="n">
@@ -2322,7 +2310,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>44437</v>
       </c>
       <c r="B36" t="n">
@@ -2375,7 +2363,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>44444</v>
       </c>
       <c r="B37" t="n">
@@ -2428,7 +2416,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>44451</v>
       </c>
       <c r="B38" t="n">
@@ -2481,7 +2469,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>44458</v>
       </c>
       <c r="B39" t="n">
@@ -2534,7 +2522,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>44465</v>
       </c>
       <c r="B40" t="n">
@@ -2587,7 +2575,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>44472</v>
       </c>
       <c r="B41" t="n">
@@ -2640,7 +2628,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>44479</v>
       </c>
       <c r="B42" t="n">
@@ -2693,7 +2681,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>44486</v>
       </c>
       <c r="B43" t="n">
@@ -2746,7 +2734,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>44493</v>
       </c>
       <c r="B44" t="n">
@@ -2799,7 +2787,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>44500</v>
       </c>
       <c r="B45" t="n">
@@ -2852,7 +2840,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>44507</v>
       </c>
       <c r="B46" t="n">
@@ -2905,7 +2893,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>44514</v>
       </c>
       <c r="B47" t="n">
@@ -2958,7 +2946,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>44521</v>
       </c>
       <c r="B48" t="n">
@@ -3011,7 +2999,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>44528</v>
       </c>
       <c r="B49" t="n">
@@ -3064,7 +3052,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>44535</v>
       </c>
       <c r="B50" t="n">
@@ -3117,7 +3105,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>44542</v>
       </c>
       <c r="B51" t="n">
@@ -3170,7 +3158,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>44549</v>
       </c>
       <c r="B52" t="n">
@@ -3223,7 +3211,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>44556</v>
       </c>
       <c r="B53" t="n">
@@ -3276,7 +3264,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>44563</v>
       </c>
       <c r="B54" t="n">
@@ -3329,7 +3317,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>44570</v>
       </c>
       <c r="B55" t="n">
@@ -3382,7 +3370,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>44577</v>
       </c>
       <c r="B56" t="n">
@@ -3435,7 +3423,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>44584</v>
       </c>
       <c r="B57" t="n">
@@ -3488,7 +3476,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>44591</v>
       </c>
       <c r="B58" t="n">
@@ -3541,7 +3529,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>44598</v>
       </c>
       <c r="B59" t="n">
@@ -3594,7 +3582,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>44605</v>
       </c>
       <c r="B60" t="n">
@@ -3647,7 +3635,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>44612</v>
       </c>
       <c r="B61" t="n">
@@ -3700,7 +3688,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>44619</v>
       </c>
       <c r="B62" t="n">
@@ -3753,7 +3741,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>44626</v>
       </c>
       <c r="B63" t="n">
@@ -3806,7 +3794,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>44633</v>
       </c>
       <c r="B64" t="n">
@@ -3859,7 +3847,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>44640</v>
       </c>
       <c r="B65" t="n">
@@ -3912,7 +3900,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>44647</v>
       </c>
       <c r="B66" t="n">
@@ -3965,7 +3953,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>44654</v>
       </c>
       <c r="B67" t="n">
@@ -4018,7 +4006,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>44661</v>
       </c>
       <c r="B68" t="n">
@@ -4071,7 +4059,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>44668</v>
       </c>
       <c r="B69" t="n">
@@ -4124,7 +4112,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>44675</v>
       </c>
       <c r="B70" t="n">
@@ -4177,7 +4165,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>44682</v>
       </c>
       <c r="B71" t="n">
@@ -4230,7 +4218,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>44689</v>
       </c>
       <c r="B72" t="n">
@@ -4283,7 +4271,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>44696</v>
       </c>
       <c r="B73" t="n">
@@ -4336,7 +4324,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>44703</v>
       </c>
       <c r="B74" t="n">
@@ -4389,7 +4377,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>44710</v>
       </c>
       <c r="B75" t="n">
@@ -4442,7 +4430,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>44717</v>
       </c>
       <c r="B76" t="n">
@@ -4495,7 +4483,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>44724</v>
       </c>
       <c r="B77" t="n">
@@ -4548,7 +4536,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>44731</v>
       </c>
       <c r="B78" t="n">
@@ -4601,7 +4589,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>44738</v>
       </c>
       <c r="B79" t="n">
@@ -4654,7 +4642,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>44745</v>
       </c>
       <c r="B80" t="n">
@@ -4707,7 +4695,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>44752</v>
       </c>
       <c r="B81" t="n">
@@ -4760,7 +4748,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>44759</v>
       </c>
       <c r="B82" t="n">
@@ -4813,7 +4801,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>44766</v>
       </c>
       <c r="B83" t="n">
@@ -4866,7 +4854,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>44773</v>
       </c>
       <c r="B84" t="n">
@@ -4919,7 +4907,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>44780</v>
       </c>
       <c r="B85" t="n">
@@ -4972,7 +4960,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>44787</v>
       </c>
       <c r="B86" t="n">
@@ -5025,7 +5013,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>44794</v>
       </c>
       <c r="B87" t="n">
@@ -5078,7 +5066,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>44801</v>
       </c>
       <c r="B88" t="n">
@@ -5131,7 +5119,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>44808</v>
       </c>
       <c r="B89" t="n">
@@ -5184,7 +5172,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>44815</v>
       </c>
       <c r="B90" t="n">
@@ -5237,7 +5225,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>44822</v>
       </c>
       <c r="B91" t="n">
@@ -5290,7 +5278,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>44829</v>
       </c>
       <c r="B92" t="n">
@@ -5343,7 +5331,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>44836</v>
       </c>
       <c r="B93" t="n">
@@ -5396,7 +5384,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>44843</v>
       </c>
       <c r="B94" t="n">
@@ -5449,7 +5437,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>44850</v>
       </c>
       <c r="B95" t="n">
@@ -5502,7 +5490,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>44857</v>
       </c>
       <c r="B96" t="n">
@@ -5555,7 +5543,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>44864</v>
       </c>
       <c r="B97" t="n">
@@ -5608,7 +5596,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>44871</v>
       </c>
       <c r="B98" t="n">
@@ -5661,7 +5649,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>44878</v>
       </c>
       <c r="B99" t="n">
@@ -5714,7 +5702,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>44885</v>
       </c>
       <c r="B100" t="n">
@@ -5767,7 +5755,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>44892</v>
       </c>
       <c r="B101" t="n">
@@ -5820,7 +5808,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>44899</v>
       </c>
       <c r="B102" t="n">
@@ -5873,7 +5861,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>44906</v>
       </c>
       <c r="B103" t="n">
@@ -5926,7 +5914,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>44913</v>
       </c>
       <c r="B104" t="n">
@@ -5979,7 +5967,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>44920</v>
       </c>
       <c r="B105" t="n">
@@ -6032,7 +6020,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>44927</v>
       </c>
       <c r="B106" t="n">
@@ -6085,7 +6073,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>44934</v>
       </c>
       <c r="B107" t="n">
@@ -6138,7 +6126,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>44941</v>
       </c>
       <c r="B108" t="n">
@@ -6191,7 +6179,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>44948</v>
       </c>
       <c r="B109" t="n">
@@ -6244,7 +6232,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>44955</v>
       </c>
       <c r="B110" t="n">
@@ -6297,7 +6285,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>44962</v>
       </c>
       <c r="B111" t="n">
@@ -6350,7 +6338,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>44969</v>
       </c>
       <c r="B112" t="n">
@@ -6403,7 +6391,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>44976</v>
       </c>
       <c r="B113" t="n">
@@ -6456,7 +6444,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>44983</v>
       </c>
       <c r="B114" t="n">
@@ -6509,7 +6497,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>44990</v>
       </c>
       <c r="B115" t="n">
@@ -6562,7 +6550,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>44997</v>
       </c>
       <c r="B116" t="n">
@@ -6615,7 +6603,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>45004</v>
       </c>
       <c r="B117" t="n">
@@ -6668,7 +6656,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>45011</v>
       </c>
       <c r="B118" t="n">
@@ -6721,7 +6709,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>45018</v>
       </c>
       <c r="B119" t="n">
@@ -6774,7 +6762,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>45025</v>
       </c>
       <c r="B120" t="n">
@@ -6827,7 +6815,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>45032</v>
       </c>
       <c r="B121" t="n">
@@ -6880,7 +6868,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>45039</v>
       </c>
       <c r="B122" t="n">
@@ -6933,7 +6921,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>45046</v>
       </c>
       <c r="B123" t="n">
@@ -6986,7 +6974,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>45053</v>
       </c>
       <c r="B124" t="n">
@@ -7039,7 +7027,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>45060</v>
       </c>
       <c r="B125" t="n">
@@ -7092,7 +7080,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>45067</v>
       </c>
       <c r="B126" t="n">
@@ -7145,7 +7133,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>45074</v>
       </c>
       <c r="B127" t="n">
@@ -7198,7 +7186,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>45081</v>
       </c>
       <c r="B128" t="n">
@@ -7251,7 +7239,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>45088</v>
       </c>
       <c r="B129" t="n">
@@ -7304,7 +7292,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>45095</v>
       </c>
       <c r="B130" t="n">
@@ -7357,7 +7345,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>45102</v>
       </c>
       <c r="B131" t="n">
@@ -7410,7 +7398,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>45109</v>
       </c>
       <c r="B132" t="n">
@@ -7463,7 +7451,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>45116</v>
       </c>
       <c r="B133" t="n">
@@ -7516,7 +7504,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>45123</v>
       </c>
       <c r="B134" t="n">
@@ -7569,7 +7557,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>45130</v>
       </c>
       <c r="B135" t="n">
@@ -7622,7 +7610,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>45137</v>
       </c>
       <c r="B136" t="n">
@@ -7675,7 +7663,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>45144</v>
       </c>
       <c r="B137" t="n">
@@ -7728,7 +7716,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>45151</v>
       </c>
       <c r="B138" t="n">
@@ -7781,7 +7769,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>45158</v>
       </c>
       <c r="B139" t="n">
@@ -7834,7 +7822,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>45165</v>
       </c>
       <c r="B140" t="n">
@@ -7887,7 +7875,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>45172</v>
       </c>
       <c r="B141" t="n">
@@ -7940,7 +7928,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>45179</v>
       </c>
       <c r="B142" t="n">
@@ -7993,7 +7981,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>45186</v>
       </c>
       <c r="B143" t="n">
@@ -8046,7 +8034,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>45193</v>
       </c>
       <c r="B144" t="n">
@@ -8099,7 +8087,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>45200</v>
       </c>
       <c r="B145" t="n">
@@ -8152,7 +8140,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>45207</v>
       </c>
       <c r="B146" t="n">
@@ -8205,7 +8193,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>45214</v>
       </c>
       <c r="B147" t="n">
@@ -8258,7 +8246,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>45221</v>
       </c>
       <c r="B148" t="n">
@@ -8311,7 +8299,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>45228</v>
       </c>
       <c r="B149" t="n">
@@ -8364,7 +8352,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>45235</v>
       </c>
       <c r="B150" t="n">
@@ -8417,7 +8405,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>45242</v>
       </c>
       <c r="B151" t="n">
@@ -8470,7 +8458,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>45249</v>
       </c>
       <c r="B152" t="n">
@@ -8523,7 +8511,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>45256</v>
       </c>
       <c r="B153" t="n">
@@ -8576,7 +8564,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>45263</v>
       </c>
       <c r="B154" t="n">
@@ -8629,7 +8617,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>45270</v>
       </c>
       <c r="B155" t="n">
@@ -8682,7 +8670,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>45277</v>
       </c>
       <c r="B156" t="n">
@@ -8735,7 +8723,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>45284</v>
       </c>
       <c r="B157" t="n">
@@ -8788,7 +8776,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>45291</v>
       </c>
       <c r="B158" t="n">
@@ -8841,7 +8829,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>45298</v>
       </c>
       <c r="B159" t="n">
@@ -8894,7 +8882,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>45305</v>
       </c>
       <c r="B160" t="n">
@@ -8947,7 +8935,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>45312</v>
       </c>
       <c r="B161" t="n">
@@ -9000,7 +8988,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>45319</v>
       </c>
       <c r="B162" t="n">
@@ -9053,7 +9041,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>45326</v>
       </c>
       <c r="B163" t="n">
@@ -9106,7 +9094,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>45333</v>
       </c>
       <c r="B164" t="n">
@@ -9159,7 +9147,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>45340</v>
       </c>
       <c r="B165" t="n">
@@ -9212,7 +9200,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>45347</v>
       </c>
       <c r="B166" t="n">
@@ -9265,7 +9253,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>45354</v>
       </c>
       <c r="B167" t="n">
@@ -9318,7 +9306,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>45361</v>
       </c>
       <c r="B168" t="n">
@@ -9371,7 +9359,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>45368</v>
       </c>
       <c r="B169" t="n">
@@ -9424,7 +9412,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>45375</v>
       </c>
       <c r="B170" t="n">
@@ -9477,7 +9465,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>45382</v>
       </c>
       <c r="B171" t="n">
@@ -9530,7 +9518,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>45389</v>
       </c>
       <c r="B172" t="n">
@@ -9583,7 +9571,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>45396</v>
       </c>
       <c r="B173" t="n">
@@ -9636,7 +9624,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>45403</v>
       </c>
       <c r="B174" t="n">
@@ -9689,7 +9677,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>45410</v>
       </c>
       <c r="B175" t="n">
@@ -9742,7 +9730,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>45417</v>
       </c>
       <c r="B176" t="n">
@@ -9795,7 +9783,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>45424</v>
       </c>
       <c r="B177" t="n">
@@ -9848,7 +9836,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>45431</v>
       </c>
       <c r="B178" t="n">
@@ -9901,7 +9889,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>45438</v>
       </c>
       <c r="B179" t="n">
@@ -9954,7 +9942,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>45445</v>
       </c>
       <c r="B180" t="n">
@@ -10007,7 +9995,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>45452</v>
       </c>
       <c r="B181" t="n">
@@ -10060,7 +10048,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>45459</v>
       </c>
       <c r="B182" t="n">
@@ -10113,7 +10101,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>45466</v>
       </c>
       <c r="B183" t="n">
@@ -10166,7 +10154,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>45473</v>
       </c>
       <c r="B184" t="n">
@@ -10219,7 +10207,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>45480</v>
       </c>
       <c r="B185" t="n">
@@ -10272,7 +10260,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>45487</v>
       </c>
       <c r="B186" t="n">
@@ -10325,7 +10313,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>45494</v>
       </c>
       <c r="B187" t="n">
@@ -10378,7 +10366,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>45501</v>
       </c>
       <c r="B188" t="n">
@@ -10431,7 +10419,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>45508</v>
       </c>
       <c r="B189" t="n">
@@ -10484,7 +10472,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>45515</v>
       </c>
       <c r="B190" t="n">
@@ -10537,7 +10525,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>45522</v>
       </c>
       <c r="B191" t="n">
@@ -10590,7 +10578,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>45529</v>
       </c>
       <c r="B192" t="n">
@@ -10643,7 +10631,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>45536</v>
       </c>
       <c r="B193" t="n">
@@ -10696,7 +10684,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>45543</v>
       </c>
       <c r="B194" t="n">
@@ -10749,7 +10737,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>45550</v>
       </c>
       <c r="B195" t="n">
@@ -10802,7 +10790,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>45557</v>
       </c>
       <c r="B196" t="n">
@@ -10855,7 +10843,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>45564</v>
       </c>
       <c r="B197" t="n">
@@ -10908,7 +10896,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>45571</v>
       </c>
       <c r="B198" t="n">
@@ -10961,7 +10949,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>45578</v>
       </c>
       <c r="B199" t="n">
@@ -11014,7 +11002,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>45585</v>
       </c>
       <c r="B200" t="n">
@@ -11067,7 +11055,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>45592</v>
       </c>
       <c r="B201" t="n">
@@ -11120,7 +11108,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>45599</v>
       </c>
       <c r="B202" t="n">
@@ -11173,7 +11161,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>45606</v>
       </c>
       <c r="B203" t="n">
@@ -11226,7 +11214,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>45613</v>
       </c>
       <c r="B204" t="n">
@@ -11279,7 +11267,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>45620</v>
       </c>
       <c r="B205" t="n">
@@ -11332,7 +11320,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>45627</v>
       </c>
       <c r="B206" t="n">
@@ -11385,7 +11373,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>45634</v>
       </c>
       <c r="B207" t="n">
@@ -11438,7 +11426,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>45641</v>
       </c>
       <c r="B208" t="n">
@@ -11491,7 +11479,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>45648</v>
       </c>
       <c r="B209" t="n">
@@ -11544,7 +11532,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>45655</v>
       </c>
       <c r="B210" t="n">
@@ -11597,7 +11585,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>45662</v>
       </c>
       <c r="B211" t="n">
@@ -11650,7 +11638,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>45669</v>
       </c>
       <c r="B212" t="n">
@@ -11703,7 +11691,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>45676</v>
       </c>
       <c r="B213" t="n">
@@ -11756,7 +11744,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>45683</v>
       </c>
       <c r="B214" t="n">
@@ -11809,7 +11797,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>45690</v>
       </c>
       <c r="B215" t="n">
@@ -11862,7 +11850,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>45697</v>
       </c>
       <c r="B216" t="n">
@@ -11915,7 +11903,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>45704</v>
       </c>
       <c r="B217" t="n">
@@ -11968,7 +11956,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>45711</v>
       </c>
       <c r="B218" t="n">
@@ -12021,7 +12009,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>45718</v>
       </c>
       <c r="B219" t="n">
@@ -12074,7 +12062,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>45725</v>
       </c>
       <c r="B220" t="n">
@@ -12127,7 +12115,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>45732</v>
       </c>
       <c r="B221" t="n">
@@ -12180,7 +12168,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>45739</v>
       </c>
       <c r="B222" t="n">
@@ -12233,7 +12221,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>45746</v>
       </c>
       <c r="B223" t="n">
@@ -12286,7 +12274,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>45753</v>
       </c>
       <c r="B224" t="n">
@@ -12339,7 +12327,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>45760</v>
       </c>
       <c r="B225" t="n">
@@ -12392,7 +12380,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>45767</v>
       </c>
       <c r="B226" t="n">
@@ -12445,7 +12433,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>45774</v>
       </c>
       <c r="B227" t="n">
@@ -12498,7 +12486,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>45781</v>
       </c>
       <c r="B228" t="n">
@@ -12551,7 +12539,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>45788</v>
       </c>
       <c r="B229" t="n">
@@ -12604,7 +12592,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>45795</v>
       </c>
       <c r="B230" t="n">
@@ -12657,7 +12645,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>45802</v>
       </c>
       <c r="B231" t="n">
@@ -12710,7 +12698,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>45809</v>
       </c>
       <c r="B232" t="n">
@@ -12763,7 +12751,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>45816</v>
       </c>
       <c r="B233" t="n">
@@ -12816,7 +12804,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>45823</v>
       </c>
       <c r="B234" t="n">
@@ -12869,7 +12857,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>45830</v>
       </c>
       <c r="B235" t="n">
@@ -12922,7 +12910,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>45837</v>
       </c>
       <c r="B236" t="n">
@@ -12975,7 +12963,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>45844</v>
       </c>
       <c r="B237" t="n">
@@ -13028,7 +13016,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="B238" t="n">
@@ -13081,7 +13069,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>45858</v>
       </c>
       <c r="B239" t="n">
@@ -13134,7 +13122,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>45865</v>
       </c>
       <c r="B240" t="n">
@@ -13187,7 +13175,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>45872</v>
       </c>
       <c r="B241" t="n">
@@ -13240,7 +13228,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>45879</v>
       </c>
       <c r="B242" t="n">
@@ -13293,7 +13281,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>45886</v>
       </c>
       <c r="B243" t="n">
@@ -13346,7 +13334,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>45893</v>
       </c>
       <c r="B244" t="n">
@@ -13399,7 +13387,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>45900</v>
       </c>
       <c r="B245" t="n">
@@ -13452,7 +13440,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>45907</v>
       </c>
       <c r="B246" t="n">
@@ -13505,7 +13493,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="n">
+      <c r="A247" s="1" t="n">
         <v>45914</v>
       </c>
       <c r="B247" t="n">
@@ -13558,7 +13546,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="n">
+      <c r="A248" s="1" t="n">
         <v>45921</v>
       </c>
       <c r="B248" t="n">
@@ -13611,7 +13599,7 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="2" t="n">
+      <c r="A249" s="1" t="n">
         <v>45928</v>
       </c>
       <c r="B249" t="n">
@@ -13664,7 +13652,7 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="2" t="n">
+      <c r="A250" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="B250" t="n">
@@ -13717,7 +13705,7 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="2" t="n">
+      <c r="A251" s="1" t="n">
         <v>45942</v>
       </c>
       <c r="B251" t="n">
@@ -13770,7 +13758,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="n">
+      <c r="A252" s="1" t="n">
         <v>45949</v>
       </c>
       <c r="B252" t="n">
@@ -13823,7 +13811,7 @@
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="2" t="n">
+      <c r="A253" s="1" t="n">
         <v>45956</v>
       </c>
       <c r="B253" t="n">
@@ -13876,7 +13864,7 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="n">
+      <c r="A254" s="1" t="n">
         <v>45963</v>
       </c>
       <c r="B254" t="n">
@@ -13929,7 +13917,7 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="2" t="n">
+      <c r="A255" s="1" t="n">
         <v>45970</v>
       </c>
       <c r="B255" t="n">
@@ -13982,7 +13970,7 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="n">
+      <c r="A256" s="1" t="n">
         <v>45977</v>
       </c>
       <c r="B256" t="n">
@@ -14035,7 +14023,7 @@
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="2" t="n">
+      <c r="A257" s="1" t="n">
         <v>45984</v>
       </c>
       <c r="B257" t="n">
@@ -14088,7 +14076,7 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="n">
+      <c r="A258" s="1" t="n">
         <v>45991</v>
       </c>
       <c r="B258" t="n">
@@ -14141,7 +14129,7 @@
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="2" t="n">
+      <c r="A259" s="1" t="n">
         <v>45998</v>
       </c>
       <c r="B259" t="n">
@@ -14194,7 +14182,7 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="2" t="n">
+      <c r="A260" s="1" t="n">
         <v>46005</v>
       </c>
       <c r="B260" t="n">
@@ -14247,7 +14235,7 @@
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="2" t="n">
+      <c r="A261" s="1" t="n">
         <v>46012</v>
       </c>
       <c r="B261" t="n">
@@ -14300,7 +14288,7 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="n">
+      <c r="A262" s="1" t="n">
         <v>46019</v>
       </c>
       <c r="B262" t="n">

</xml_diff>